<commit_message>
Sync GitHub Pages site with fixed audio
</commit_message>
<xml_diff>
--- a/docs/tabulka-radost.xlsx
+++ b/docs/tabulka-radost.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Kajik BP web\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E112788A-36B2-4163-B036-BE2D42D4B4CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{110C6F5B-4ED6-47EB-A0F2-C306D77F2585}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{F919D72D-6EEA-46E4-BD17-FBF57A672A1B}"/>
+    <workbookView xWindow="-26355" yWindow="4215" windowWidth="21600" windowHeight="11385" xr2:uid="{F919D72D-6EEA-46E4-BD17-FBF57A672A1B}"/>
   </bookViews>
   <sheets>
     <sheet name="List1" sheetId="1" r:id="rId1"/>
@@ -65,9 +65,6 @@
     <t>To/. je/. su/. per/.</t>
   </si>
   <si>
-    <t>Mám/. tě/. rád/-</t>
-  </si>
-  <si>
     <t>To/. se/. mi/. lí/- bí/-</t>
   </si>
   <si>
@@ -293,6 +290,9 @@
       </rPr>
       <t>super</t>
     </r>
+  </si>
+  <si>
+    <t>Mám/- tě/. rád/-</t>
   </si>
 </sst>
 </file>
@@ -690,7 +690,7 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B1" t="s">
         <v>0</v>
@@ -698,7 +698,7 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B2" t="s">
         <v>1</v>
@@ -706,15 +706,15 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B3" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B4" t="s">
         <v>2</v>
@@ -722,7 +722,7 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B5" t="s">
         <v>3</v>
@@ -730,7 +730,7 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B6" t="s">
         <v>4</v>
@@ -738,18 +738,18 @@
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B7" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B8" t="s">
-        <v>8</v>
+        <v>19</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
@@ -762,7 +762,7 @@
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B10" t="s">
         <v>7</v>

</xml_diff>